<commit_message>
[Data] Import coachs infos from docx file (convert to xlsx file)
</commit_message>
<xml_diff>
--- a/server/ext_num_coach.xlsx
+++ b/server/ext_num_coach.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mon Drive\Projets\Selhani\2026\Photos\Entraineurs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\samir\archifoot\server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B88C4D4C-3A6E-449A-B574-294D853D7926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E07561-F6EF-4176-837D-2F456D49E09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -159,9 +159,6 @@
     <t>E22</t>
   </si>
   <si>
-    <t>Mehdaoui Abderhamane</t>
-  </si>
-  <si>
     <t>E23</t>
   </si>
   <si>
@@ -253,6 +250,9 @@
   </si>
   <si>
     <t>E18</t>
+  </si>
+  <si>
+    <t>Mehdaoui Abderhmane</t>
   </si>
 </sst>
 </file>
@@ -363,6 +363,22 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -429,22 +445,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
     <dxf>
       <fill>
@@ -672,14 +672,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{28306622-806A-4534-AFE4-807202ADC74E}" name="Tableau1" displayName="Tableau1" ref="A1:B37" totalsRowShown="0" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{28306622-806A-4534-AFE4-807202ADC74E}" name="Tableau1" displayName="Tableau1" ref="A1:B37" totalsRowShown="0" dataDxfId="2">
   <autoFilter ref="A1:B37" xr:uid="{28306622-806A-4534-AFE4-807202ADC74E}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B37">
     <sortCondition ref="A1:A37"/>
   </sortState>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{1AA7B661-9500-44A1-A313-04F7072701B9}" name="Num" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{4465DDCF-2154-4165-88E1-95091C18347E}" name="Entraineur" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{1AA7B661-9500-44A1-A313-04F7072701B9}" name="Num" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{4465DDCF-2154-4165-88E1-95091C18347E}" name="Entraineur" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStylePreset3_Accent1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -951,10 +951,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" t="s">
         <v>71</v>
-      </c>
-      <c r="B1" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1031,7 +1031,7 @@
     </row>
     <row r="11" spans="1:2" ht="15.75">
       <c r="A11" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>34</v>
@@ -1074,63 +1074,63 @@
         <v>41</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.75">
       <c r="A17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15.75">
       <c r="A18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15.75">
       <c r="A19" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15.75">
       <c r="A20" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15.75">
       <c r="A21" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15.75">
       <c r="A22" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>53</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.75">
       <c r="A23" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="15.75">
@@ -1143,58 +1143,58 @@
     </row>
     <row r="25" spans="1:2" ht="15.75">
       <c r="A25" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="15.75">
       <c r="A26" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>59</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="15.75">
       <c r="A27" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="15.75">
       <c r="A28" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="15.75">
       <c r="A29" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>65</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="15.75">
       <c r="A30" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="15.75">
       <c r="A31" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:2">

</xml_diff>